<commit_message>
refactor: 技能按键绑定内聚 + Pilot/SkillBinding 合并为 InputBinding
- HeroData: 新增 SkillKeys 列，按键与技能列表一一对应
- SkillInfo: 新增 key 字段，按键绑定随技能数据一起装载
- SkillLauncher.Load: 新增 key 参数
- HeroPrefab/EnemyPrefab: 装载技能时传入 key（敌人 key=0）
- 移除 SkillBindingData 表及相关生成代码
- Pilot + SkillBinding 合并为 InputBinding，统一处理移动意图和技能触发
- Stage.cs: tabs 缩进统一为 spaces

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Config/Datas/HeroData.xlsx
+++ b/Config/Datas/HeroData.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="18.75"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -525,12 +525,17 @@
           <t>Skills</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>SkillKeys</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>BornPipelines</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>DeathPipelines</t>
         </is>
@@ -572,12 +577,17 @@
           <t>(list#sep=|),int</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>(list#sep=|),int</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>(list#sep=|),int</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>(list#sep=|),int</t>
         </is>
@@ -619,12 +629,17 @@
           <t>技能列表</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>技能按键列表（与 Skills 一一对应）</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
         <is>
           <t>出生管线</t>
         </is>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>死亡管线</t>
         </is>
@@ -650,10 +665,15 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>10001|10002|10003|10004|10010</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n">
+          <t>10001|10002|10003|10004|10010|10020|10030</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1002|1002|1002|1002|0|1003|1004</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n">
         <v>10010</v>
       </c>
     </row>
@@ -677,10 +697,15 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>10001|10002|10003|10004|10010</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="n">
+          <t>10001|10002|10003|10004|10010|10020|10030</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1002|1002|1002|1002|0|1003|1004</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n">
         <v>10010</v>
       </c>
     </row>

</xml_diff>